<commit_message>
Update SOX yfinance proxy through latest tracking date
</commit_message>
<xml_diff>
--- a/sox_daily_tracking_log.xlsx
+++ b/sox_daily_tracking_log.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R30"/>
+  <dimension ref="A1:S34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -518,6 +518,11 @@
       <c r="R1" t="inlineStr">
         <is>
           <t>Last_Updated_Time</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>YF_Index_Price</t>
         </is>
       </c>
     </row>
@@ -1294,7 +1299,7 @@
         <v>0.5422695929298591</v>
       </c>
       <c r="L30" t="n">
-        <v>1.034428591314902</v>
+        <v>1.034428591314903</v>
       </c>
       <c r="M30" t="n">
         <v>1.02112118796327</v>
@@ -1312,6 +1317,209 @@
         <is>
           <t>2026-07-03 16:19:48</t>
         </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>12626.221</v>
+      </c>
+      <c r="C31" t="n">
+        <v>51.54583</v>
+      </c>
+      <c r="D31" t="n">
+        <v>26.19895178082191</v>
+      </c>
+      <c r="E31" t="n">
+        <v>49.81575658664247</v>
+      </c>
+      <c r="F31" t="n">
+        <v>25.63538962820493</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Jul 02, 2026</t>
+        </is>
+      </c>
+      <c r="H31" t="n">
+        <v>74.38</v>
+      </c>
+      <c r="J31" t="n">
+        <v>1.730073413357538</v>
+      </c>
+      <c r="K31" t="n">
+        <v>0.5635621526169814</v>
+      </c>
+      <c r="L31" t="n">
+        <v>1.034729441684751</v>
+      </c>
+      <c r="M31" t="n">
+        <v>1.021983756080576</v>
+      </c>
+      <c r="N31" t="n">
+        <v>-22.83417</v>
+      </c>
+      <c r="P31" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>0</v>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>2026-07-04 10:00:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>12626.221</v>
+      </c>
+      <c r="C32" t="n">
+        <v>51.54583</v>
+      </c>
+      <c r="D32" t="n">
+        <v>26.18112978082192</v>
+      </c>
+      <c r="E32" t="n">
+        <v>49.81575658664247</v>
+      </c>
+      <c r="F32" t="n">
+        <v>25.60753883662741</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Jul 02, 2026</t>
+        </is>
+      </c>
+      <c r="H32" t="n">
+        <v>74.38</v>
+      </c>
+      <c r="J32" t="n">
+        <v>1.730073413357538</v>
+      </c>
+      <c r="K32" t="n">
+        <v>0.573590944194514</v>
+      </c>
+      <c r="L32" t="n">
+        <v>1.034729441684751</v>
+      </c>
+      <c r="M32" t="n">
+        <v>1.022399299981695</v>
+      </c>
+      <c r="N32" t="n">
+        <v>-22.83417</v>
+      </c>
+      <c r="P32" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>0</v>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>2026-07-05 10:00:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>12626.221</v>
+      </c>
+      <c r="C33" t="n">
+        <v>51.54583</v>
+      </c>
+      <c r="D33" t="n">
+        <v>26.16361257534247</v>
+      </c>
+      <c r="E33" t="n">
+        <v>49.81575658664247</v>
+      </c>
+      <c r="F33" t="n">
+        <v>25.57974849467187</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Jul 02, 2026</t>
+        </is>
+      </c>
+      <c r="H33" t="n">
+        <v>74.38</v>
+      </c>
+      <c r="J33" t="n">
+        <v>1.730073413357538</v>
+      </c>
+      <c r="K33" t="n">
+        <v>0.5838640806705939</v>
+      </c>
+      <c r="L33" t="n">
+        <v>1.034729441684751</v>
+      </c>
+      <c r="M33" t="n">
+        <v>1.022825247120479</v>
+      </c>
+      <c r="N33" t="n">
+        <v>-22.83417</v>
+      </c>
+      <c r="P33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>0</v>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>2026-07-06 10:00:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>49.15125264480251</v>
+      </c>
+      <c r="F34" t="n">
+        <v>25.11654259125032</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Jul 06, 2026</t>
+        </is>
+      </c>
+      <c r="H34" t="n">
+        <v>71.37</v>
+      </c>
+      <c r="P34" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>0</v>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>2026-07-08 09:07:35</t>
+        </is>
+      </c>
+      <c r="S34" t="n">
+        <v>12300.516</v>
       </c>
     </row>
   </sheetData>

</xml_diff>